<commit_message>
TV3: module data (Cloud SQL HA pgvector, GCS workspace, Redis HA, Cloud Tasks, Pub/Sub), RLS isolation test, bao gia 5 component, so do slide 6-7
- terraform/modules/data: PG16 regional HA, IAM auth, pgaudit; GCS CMEK + quyen KMS cho GCS agent;
  Redis STANDARD_HA 5 GB co AUTH/TLS; 2 hang doi Cloud Tasks; Pub/Sub + DLQ, Cloud Scheduler; staging DB
- tv3_data: schema pgvector + Row-Level Security, kiem thu co lap user A/B (7/7 PASS), ban ghi SKU gia
- baogia: 14 dong TV3 (890.86 USD/thang), bang chung E30-E37
- slides: so do Slide 6, 7 va noi dung Slide 6, 7, 12 (phan du lieu)
- TV3_LamHoangPhuc.md: bao cao ca nhan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/baogia/Gxx_baogia.xlsx
+++ b/baogia/Gxx_baogia.xlsx
@@ -7,7 +7,7 @@
     <sheet name="BangChung" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">BaoGia!$A$1:$E$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">BaoGia!$A$1:$E$46</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E46"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -517,542 +517,695 @@
         <v>connectors</v>
       </c>
       <c r="B7" t="str">
-        <v>Connectors Google Workspace, M365, Notion, Jira, Confluence</v>
+        <v>Gọi API SaaS (Gmail, Drive, Calendar, Outlook, OneDrive, SharePoint, Teams, Notion, Jira, Confluence) bằng OAuth ủy nhiệm của từng user</v>
       </c>
       <c r="C7" t="str">
-        <v>CHỜ TV3 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
+        <v>Phí gọi API của Google Workspace, Microsoft Graph, Notion, Jira, Confluence nằm trong license SaaS tập đoàn đang trả; connector worker chạy trên GKE nằm trong dòng compute, lưu lượng ra SaaS qua Cloud NAT nằm trong dòng network. Rate limit từng SaaS theo link bằng chứng; ~20.000 lượt gọi/ngày</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>https://developers.google.com/workspace/gmail/api/reference/quota; https://learn.microsoft.com/en-us/graph/throttling; https://developer.atlassian.com/cloud/jira/platform/rate-limiting/</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>database</v>
+        <v>connectors</v>
       </c>
       <c r="B8" t="str">
-        <v>Cloud SQL PostgreSQL HA (regional) cho metadata, lịch sử chat</v>
+        <v>Pub/Sub nhận thông báo thay đổi (Gmail/Drive watch, webhook M365/Jira/Confluence/Notion) cho đồng bộ index theo sự kiện</v>
       </c>
       <c r="C8" t="str">
-        <v>CHỜ TV3 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D8" t="str">
-        <v/>
+        <v>Pub/Sub Message Delivery, SKU 027D-B6C7-CCA2: 2,2 triệu event/tháng × 1 KB × 2 (publish + delivery) = 4.4 GB = 0.0043 TiB × 40 USD/TiB, cộng lưu 1 ngày ~0,1 GB × 0,27 USD (F9EB-D3E1-ABDF). Tính toàn bộ theo đơn giá niêm yết</v>
+      </c>
+      <c r="D8">
+        <v>0.2</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>E35; https://cloud.google.com/pubsub/pricing</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>vector_db</v>
+        <v>connectors</v>
       </c>
       <c r="B9" t="str">
-        <v>pgvector trên Cloud SQL, lọc kết quả theo ACL gốc</v>
+        <v>Cloud Scheduler: delta sync 15 phút/lần trong giờ hành chính cho 5 nhóm connector</v>
       </c>
       <c r="C9" t="str">
-        <v>CHỜ TV3 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
+        <v>Cloud Scheduler Jobs, SKU A5D6-43A2-28A7: 5 job × 0.1 USD/job-tháng (0,003225806 USD/job-ngày × 31)</v>
+      </c>
+      <c r="D9">
+        <v>0.5</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>E36; https://cloud.google.com/scheduler/pricing</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>object_storage</v>
+        <v>connectors</v>
       </c>
       <c r="B10" t="str">
-        <v>GCS workspace riêng từng user (prefix + CMEK, lifecycle)</v>
+        <v>Bucket tạm connector-ingest (file tải từ Drive/SharePoint để tách chunk, tự xóa sau 7 ngày, CMEK)</v>
       </c>
       <c r="C10" t="str">
-        <v>CHỜ TV3 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D10" t="str">
-        <v/>
+        <v>GCS Standard Singapore: 15 GB-tháng × 0.02 USD + 150.000 thao tác ghi × 0.000005 USD (SKU 76BA-5CAD-4338, 4DBF-185F-A415)</v>
+      </c>
+      <c r="D10">
+        <v>1.05</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>E32; https://cloud.google.com/storage/pricing</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>cache_queue</v>
+        <v>database</v>
       </c>
       <c r="B11" t="str">
-        <v>Memorystore Redis HA + Cloud Tasks cho agent chạy nền</v>
+        <v>Cloud SQL PostgreSQL 16 Regional HA (primary + standby khác zone, failover tự động): user, ACL, lịch sử chat 12 tháng, memory, metadata workspace</v>
       </c>
       <c r="C11" t="str">
-        <v>CHỜ TV3 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D11" t="str">
-        <v/>
+        <v>db-custom-4-16384, asia-southeast1, REGIONAL (multi-AZ): (4 vCPU × 0.1156 + 16 GB × 0.0196) = 0.776 USD/giờ × 730 giờ = 566.48 USD, committed use 1 năm trả 75% (giảm 25%, SKU B4F3-4753-84D8). SKU 0152-2835-C929, 37B4-B2B7-C640</v>
+      </c>
+      <c r="D11">
+        <v>424.86</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>E30; E31; https://cloud.google.com/sql/pricing</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>sandbox</v>
+        <v>database</v>
       </c>
       <c r="B12" t="str">
-        <v>GKE Sandbox node pool (gVisor) chạy code của agent</v>
+        <v>Ổ SSD Cloud SQL Regional HA 200 GB (chat 12 tháng ~84 GB, vector ~8 GB, memory + metadata ~4 GB, ×1,5 WAL/bloat, dư IOPS)</v>
       </c>
       <c r="C12" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
+        <v>Regional Standard storage Singapore, SKU 83A6-DA61-7797: 200 GB × 0.476 USD/GB-tháng (giá regional đã gồm bản sao ở zone standby). Tự tăng tối đa 500 GB</v>
+      </c>
+      <c r="D12">
+        <v>95.2</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>E30; https://cloud.google.com/sql/pricing</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>authn</v>
+        <v>database</v>
       </c>
       <c r="B13" t="str">
-        <v>SSO tập đoàn (OIDC/SAML) + MFA</v>
+        <v>Cloud SQL staging (môi trường staging): zonal, chỉ bật giờ hành chính bằng Cloud Scheduler</v>
       </c>
       <c r="C13" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D13" t="str">
-        <v/>
+        <v>db-custom-1-3840 zonal: (1 × 0.0578 + 3.75 × 0.0098) × 220 giờ = 20.8 USD; SSD 20 GB × 0.238 = 4.76 USD; 2 job Scheduler bật/tắt × 0.1 USD (SKU DE86-B401-E60F, EF83-F6A8-8EA7, 45B3-606F-EE91, A5D6-43A2-28A7)</v>
+      </c>
+      <c r="D13">
+        <v>25.76</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>E30; E36; https://cloud.google.com/sql/pricing</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>authz</v>
+        <v>vector_db</v>
       </c>
       <c r="B14" t="str">
-        <v>RBAC/ABAC, ACL tài liệu, scope OAuth tối thiểu</v>
+        <v>pgvector (HNSW, 768 chiều) trong Cloud SQL: ~800.000 chunk knowledge base + memory, lọc theo ACL gốc bằng Row-Level Security ngay trong truy vấn ANN</v>
       </c>
       <c r="C14" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D14" t="str">
-        <v/>
+        <v>Nằm trong dòng database (Cloud SQL Regional HA ở trên): vector ~8 GB đã tính vào ổ 200 GB, HNSW index ~3 GB nằm trong RAM 16 GB. Không thuê thêm dịch vụ vector riêng; RLS lọc theo acl_principals nên user không thấy chunk mình không có quyền</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>E30; E37; https://cloud.google.com/sql/docs/postgres/work-with-vectors</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>secrets_kms</v>
+        <v>object_storage</v>
       </c>
       <c r="B15" t="str">
-        <v>Cloud KMS + Secret Manager (token vault OAuth)</v>
+        <v>GCS workspace riêng từng user (prefix user-workspaces/{user_id}/, UBLA, CMEK, quota 10 GB): dữ liệu ≤ 90 ngày ở lớp Standard</v>
       </c>
       <c r="C15" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D15" t="str">
-        <v/>
+        <v>Standard Storage Singapore, SKU 76BA-5CAD-4338: 1050 GB (350 GB mới/tháng × 3 tháng; 2.000 user × ~160 MB/tháng gồm upload, file agent xuất, ảnh cấp 5, kết quả sandbox, +10% phiên bản cũ) × 0.02 USD/GB-tháng</v>
+      </c>
+      <c r="D15">
+        <v>21</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>E32; https://cloud.google.com/storage/pricing</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>governance</v>
+        <v>object_storage</v>
       </c>
       <c r="B16" t="str">
-        <v>Cloud DLP che PII, guardrail, eval gate</v>
+        <v>GCS workspace: file cũ hơn 90 ngày tự chuyển Nearline bằng lifecycle rule</v>
       </c>
       <c r="C16" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D16" t="str">
-        <v/>
+        <v>Nearline Storage Singapore, SKU 4453-FEE4-941B: 3150 GB (tháng 4-12 × 350 GB) × 0.01 USD/GB-tháng. Tổng workspace 4.200 GB = 2,1 GB/user, dưới quota 10 GB</v>
+      </c>
+      <c r="D16">
+        <v>31.5</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>E32; https://cloud.google.com/storage/pricing</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>backup_dr</v>
+        <v>object_storage</v>
       </c>
       <c r="B17" t="str">
-        <v>Backup Cloud SQL/GCS, cross-region, RTO 4h / RPO 1h</v>
+        <v>Thao tác GCS workspace: ghi, đọc, chuyển lớp lifecycle, đọc lại file Nearline</v>
       </c>
       <c r="C17" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D17" t="str">
-        <v/>
+        <v>Class A 1.32 triệu × 0.000005 + Class B 4.4 triệu × 4e-7 + chuyển lớp 440.000 object × 0.00001 + retrieval 160 GB × 0.01 USD (SKU 4DBF-185F-A415, 7870-010B-2763, 9559-D2EC-1D33, 8D92-97F6-DDF3); tính toàn bộ số thao tác theo đơn giá niêm yết</v>
+      </c>
+      <c r="D17">
+        <v>14.36</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>E32; https://cloud.google.com/storage/pricing</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>monitoring</v>
+        <v>object_storage</v>
       </c>
       <c r="B18" t="str">
-        <v>Cloud Logging/Monitoring, audit log 12 tháng, LLM observability</v>
+        <v>Bucket workspace cho staging (dữ liệu giả, tự xóa sau 30 ngày)</v>
       </c>
       <c r="C18" t="str">
-        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
-      </c>
-      <c r="D18" t="str">
-        <v/>
+        <v>Standard Storage Singapore, SKU 76BA-5CAD-4338: 50 GB × 0.02 USD/GB-tháng</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>E32; https://cloud.google.com/storage/pricing</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>compute</v>
+        <v>cache_queue</v>
       </c>
       <c r="B19" t="str">
-        <v>Phí quản lý GKE regional cluster (control plane 3 AZ, prod + staging dùng chung 1 cluster)</v>
+        <v>Memorystore for Redis Standard HA 5 GB (primary + replica khác zone, failover tự động): phiên, ngữ cảnh hội thoại, cache RAG, bộ đếm quota, cờ hủy tác vụ agent</v>
       </c>
       <c r="C19" t="str">
-        <v>GKE Regional Kubernetes Clusters, SKU B561-BFBD-1264: 1 cluster × 730 giờ × 0.1 USD/giờ. Staging chạy trong cùng cluster (namespace + node pool riêng) nên không thêm phí cluster</v>
+        <v>Redis Capacity Standard M2 Singapore, SKU A728-AD0D-27B4: 5 GB × 730 giờ × 0.075 USD/GB-giờ. Chọn 5 GB vì bậc M2 rẻ hơn: 4 GB bậc M1 = 4 × 730 × 0.114 = 332.88 USD. Staging dùng Redis container trên node staging, nằm trong compute</v>
       </c>
       <c r="D19">
-        <v>73</v>
+        <v>273.75</v>
       </c>
       <c r="E19" t="str">
-        <v>E01; https://cloud.google.com/kubernetes-engine/pricing</v>
+        <v>E33; https://cloud.google.com/memorystore/docs/redis/pricing</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>compute</v>
+        <v>cache_queue</v>
       </c>
       <c r="B20" t="str">
-        <v>Node pool app production, phần nền 24/7: web/API, LLM gateway, orchestrator, connector &amp; agent workers</v>
+        <v>Cloud Tasks: hàng đợi agent chạy nền cấp 4 (retry tối đa 10 phút) và hàng đợi đồng bộ connector</v>
       </c>
       <c r="C20" t="str">
-        <v>e2-standard-4 (4 vCPU, 16 GB), asia-southeast1, 3 node (1 node/zone × 3 zone, multi-AZ) × 730 giờ × 0.104159 USD/giờ. Committed use 1 năm cho 12 vCPU + 48 GB: 4 × 0.016952865 + 16 × 0.002271742 (SKU AA47-6F66-D143, C0B6-DC5E-4BD8)</v>
+        <v>Cloud Tasks Operations, SKU 378A-D762-1F74: 4.2 triệu operation (132.000 tác vụ agent × 6 bước × 2 = 1,58 triệu; sync theo webhook 2,2 triệu; delta tick 0,35 triệu) × 0.4 USD/triệu, tính toàn bộ theo đơn giá niêm yết</v>
       </c>
       <c r="D20">
-        <v>228.11</v>
+        <v>1.68</v>
       </c>
       <c r="E20" t="str">
-        <v>E02; https://cloud.google.com/compute/vm-instance-pricing</v>
+        <v>E34; https://cloud.google.com/tasks/pricing</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>compute</v>
+        <v>sandbox</v>
       </c>
       <c r="B21" t="str">
-        <v>Node pool app production, scale-out giờ cao điểm (autoscaler 1 → 2 node/zone)</v>
+        <v>GKE Sandbox node pool (gVisor) chạy code của agent</v>
       </c>
       <c r="C21" t="str">
-        <v>e2-standard-4 on-demand, asia-southeast1, +3 node (1 node/zone) × 220 giờ hành chính × 0.165332 USD/giờ = 4 × 0.02690931 + 16 × 0.00360594 (SKU 7102-B9AA-2ACF, E277-7DC2-2C7D). Ngoài giờ scale về 3 node</v>
-      </c>
-      <c r="D21">
-        <v>109.12</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
       </c>
       <c r="E21" t="str">
-        <v>E03; https://cloud.google.com/compute/vm-instance-pricing</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>compute</v>
+        <v>authn</v>
       </c>
       <c r="B22" t="str">
-        <v>Node pool staging (môi trường staging): 1 node Spot, chạy giờ hành chính, ngoài giờ scale về 0</v>
+        <v>SSO tập đoàn (OIDC/SAML) + MFA</v>
       </c>
       <c r="C22" t="str">
-        <v>e2-standard-4 Spot, asia-southeast1-a, 1 node × 220 giờ × 0.099224 USD/giờ = 4 × 0.01615 + 16 × 0.002164 (SKU 7217-D10E-E65B, 32B3-29BC-0D1E, giá Spot ngày 2026-10-16)</v>
-      </c>
-      <c r="D22">
-        <v>21.83</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
       </c>
       <c r="E22" t="str">
-        <v>E04; https://cloud.google.com/compute/vm-instance-pricing</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>compute</v>
+        <v>authz</v>
       </c>
       <c r="B23" t="str">
-        <v>Boot disk cho node app và staging</v>
+        <v>RBAC/ABAC, ACL tài liệu, scope OAuth tối thiểu</v>
       </c>
       <c r="C23" t="str">
-        <v>PD Standard, asia-southeast1, SKU 0572-568A-4FC4: 50 GB × (3 node 24/7 + 4 node × 220/730) = 210.3 GB-tháng × 0.044 USD</v>
-      </c>
-      <c r="D23">
-        <v>9.25</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
       </c>
       <c r="E23" t="str">
-        <v>E05; https://cloud.google.com/compute/disks-image-pricing</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>load_balancer</v>
+        <v>secrets_kms</v>
       </c>
       <c r="B24" t="str">
-        <v>Global External Application Load Balancer (anycast, đa zone, TLS 1.2+, chứng chỉ Google-managed) trước GKE Gateway</v>
+        <v>Cloud KMS + Secret Manager (token vault OAuth)</v>
       </c>
       <c r="C24" t="str">
-        <v>Forwarding rule global, SKU DEE3-C42E-3E4D: mức tối thiểu cho tới 5 rule (HTTPS + redirect HTTP) × 730 giờ × 0.025 USD/giờ. LB là dịch vụ managed, không có SPOF (HA)</v>
-      </c>
-      <c r="D24">
-        <v>18.25</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
       </c>
       <c r="E24" t="str">
-        <v>E06; https://cloud.google.com/vpc/network-pricing</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>load_balancer</v>
+        <v>governance</v>
       </c>
       <c r="B25" t="str">
-        <v>Data processing của Load Balancer tại Singapore (vào + ra)</v>
+        <v>Cloud DLP che PII, guardrail, eval gate</v>
       </c>
       <c r="C25" t="str">
-        <v>SKU 17FF-00DE-2217 / A9BA-43D3-25AD: (70 GB vào + 200 GB ra) × 0.009 USD/GB. Vào: 1,1 triệu request/tháng × 20 KB + upload file; ra: response stream + asset + file DOCX/XLSX/PPTX</v>
-      </c>
-      <c r="D25">
-        <v>2.43</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
       </c>
       <c r="E25" t="str">
-        <v>E06; https://cloud.google.com/vpc/network-pricing</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>network</v>
+        <v>backup_dr</v>
       </c>
       <c r="B26" t="str">
-        <v>Cloud NAT gateway cho node private gọi API SaaS connectors (kiểm soát egress)</v>
+        <v>Backup Cloud SQL/GCS, cross-region, RTO 4h / RPO 1h</v>
       </c>
       <c r="C26" t="str">
-        <v>SKU 32E2-4EFC-EF9F: 0.0014 USD/VM-giờ × 5260 VM-giờ (app 3×730 + 3×220, staging 1×220, sandbox 3×730). Vertex AI đi qua Private Google Access, không qua NAT</v>
-      </c>
-      <c r="D26">
-        <v>7.36</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
       </c>
       <c r="E26" t="str">
-        <v>E07; https://cloud.google.com/nat/pricing</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>network</v>
+        <v>monitoring</v>
       </c>
       <c r="B27" t="str">
-        <v>IP public của Cloud NAT (IP cố định để SaaS whitelist)</v>
+        <v>Cloud Logging/Monitoring, audit log 12 tháng, LLM observability</v>
       </c>
       <c r="C27" t="str">
-        <v>SKU 8515-9425-D2CE: 1 IP × 730 giờ × 0.005 USD/giờ</v>
-      </c>
-      <c r="D27">
-        <v>3.65</v>
+        <v>CHỜ TV4 điền: dịch vụ/SKU, region, đơn giá × số lượng</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
       </c>
       <c r="E27" t="str">
-        <v>E07; https://cloud.google.com/nat/pricing</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>network</v>
+        <v>compute</v>
       </c>
       <c r="B28" t="str">
-        <v>Dữ liệu qua Cloud NAT: gọi API Google Workspace, M365, Notion, Jira, Confluence và đồng bộ index</v>
+        <v>Phí quản lý GKE regional cluster (control plane 3 AZ, prod + staging dùng chung 1 cluster)</v>
       </c>
       <c r="C28" t="str">
-        <v>SKU 015F-5732-FFF0: 300 GB/tháng (vào + ra) × 0.045 USD/GB</v>
+        <v>GKE Regional Kubernetes Clusters, SKU B561-BFBD-1264: 1 cluster × 730 giờ × 0.1 USD/giờ. Staging chạy trong cùng cluster (namespace + node pool riêng) nên không thêm phí cluster</v>
       </c>
       <c r="D28">
-        <v>13.5</v>
+        <v>73</v>
       </c>
       <c r="E28" t="str">
-        <v>E07; https://cloud.google.com/nat/pricing</v>
+        <v>E01; https://cloud.google.com/kubernetes-engine/pricing</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>network</v>
+        <v>compute</v>
       </c>
       <c r="B29" t="str">
-        <v>Internet egress Premium Tier từ Singapore tới người dùng tại Việt Nam (APAC)</v>
+        <v>Node pool app production, phần nền 24/7: web/API, LLM gateway, orchestrator, connector &amp; agent workers</v>
       </c>
       <c r="C29" t="str">
-        <v>SKU 400E-0B94-6FB4 (Singapore → APAC, bậc 0-1 TiB): 220 GB × 0.12 USD/GB (200 GB response qua LB + 20 GB request ra SaaS)</v>
+        <v>e2-standard-4 (4 vCPU, 16 GB), asia-southeast1, 3 node (1 node/zone × 3 zone, multi-AZ) × 730 giờ × 0.104159 USD/giờ. Committed use 1 năm cho 12 vCPU + 48 GB: 4 × 0.016952865 + 16 × 0.002271742 (SKU AA47-6F66-D143, C0B6-DC5E-4BD8)</v>
       </c>
       <c r="D29">
-        <v>26.4</v>
+        <v>228.11</v>
       </c>
       <c r="E29" t="str">
-        <v>E08; https://cloud.google.com/vpc/network-pricing</v>
+        <v>E02; https://cloud.google.com/compute/vm-instance-pricing</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>network</v>
+        <v>compute</v>
       </c>
       <c r="B30" t="str">
-        <v>Lưu lượng giữa các zone (multi-AZ): pod ↔ pod, pod ↔ Cloud SQL/Redis</v>
+        <v>Node pool app production, scale-out giờ cao điểm (autoscaler 1 → 2 node/zone)</v>
       </c>
       <c r="C30" t="str">
-        <v>Inter-zone data transfer cùng region, SKU DE9E-AFBC-A15A: 200 GB × 0.01 USD/GB</v>
+        <v>e2-standard-4 on-demand, asia-southeast1, +3 node (1 node/zone) × 220 giờ hành chính × 0.165332 USD/giờ = 4 × 0.02690931 + 16 × 0.00360594 (SKU 7102-B9AA-2ACF, E277-7DC2-2C7D). Ngoài giờ scale về 3 node</v>
       </c>
       <c r="D30">
-        <v>2</v>
+        <v>109.12</v>
       </c>
       <c r="E30" t="str">
-        <v>E09; https://cloud.google.com/vpc/network-pricing</v>
+        <v>E03; https://cloud.google.com/compute/vm-instance-pricing</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>network</v>
+        <v>compute</v>
       </c>
       <c r="B31" t="str">
-        <v>Cloud Armor Standard WAF: chặn SQLi/XSS (OWASP CRS), rate limit theo IP</v>
+        <v>Node pool staging (môi trường staging): 1 node Spot, chạy giờ hành chính, ngoài giờ scale về 0</v>
       </c>
       <c r="C31" t="str">
-        <v>1 policy × 5 USD + 4 rule × 1 USD + 15 triệu request × 0.75 USD/triệu (SKU 4B13-E64F-4A2B, A321-89BD-F5BC, 1A87-DEB9-C4BE)</v>
+        <v>e2-standard-4 Spot, asia-southeast1-a, 1 node × 220 giờ × 0.099224 USD/giờ = 4 × 0.01615 + 16 × 0.002164 (SKU 7217-D10E-E65B, 32B3-29BC-0D1E, giá Spot ngày 2026-10-16)</v>
       </c>
       <c r="D31">
-        <v>20.25</v>
+        <v>21.83</v>
       </c>
       <c r="E31" t="str">
-        <v>E10; https://cloud.google.com/armor/pricing</v>
+        <v>E04; https://cloud.google.com/compute/vm-instance-pricing</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>cicd</v>
+        <v>compute</v>
       </c>
       <c r="B32" t="str">
-        <v>Cloud Build: pipeline build/test/deploy lên staging rồi production (IaC Terraform)</v>
+        <v>Boot disk cho node app và staging</v>
       </c>
       <c r="C32" t="str">
-        <v>Build time e2-standard-2, SKU A464-9020-6404: 10 service × 2 build/ngày × 22 ngày × 6 phút = 2640 phút × 0.006 USD/phút (tính toàn bộ số phút theo đơn giá niêm yết)</v>
+        <v>PD Standard, asia-southeast1, SKU 0572-568A-4FC4: 50 GB × (3 node 24/7 + 4 node × 220/730) = 210.3 GB-tháng × 0.044 USD</v>
       </c>
       <c r="D32">
-        <v>15.84</v>
+        <v>9.25</v>
       </c>
       <c r="E32" t="str">
-        <v>E11; https://cloud.google.com/build/pricing</v>
+        <v>E05; https://cloud.google.com/compute/disks-image-pricing</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>cicd</v>
+        <v>load_balancer</v>
       </c>
       <c r="B33" t="str">
-        <v>Artifact Registry: lưu container image cho staging và production</v>
+        <v>Global External Application Load Balancer (anycast, đa zone, TLS 1.2+, chứng chỉ Google-managed) trước GKE Gateway</v>
       </c>
       <c r="C33" t="str">
-        <v>SKU 8502-299A-ABAF: 30 GB (10 service × ~300 MB × giữ 10 phiên bản, cleanup policy) × 0.1 USD/GB-tháng</v>
+        <v>Forwarding rule global, SKU DEE3-C42E-3E4D: mức tối thiểu cho tới 5 rule (HTTPS + redirect HTTP) × 730 giờ × 0.025 USD/giờ. LB là dịch vụ managed, không có SPOF (HA)</v>
       </c>
       <c r="D33">
-        <v>3</v>
+        <v>18.25</v>
       </c>
       <c r="E33" t="str">
-        <v>E12; https://cloud.google.com/artifact-registry/pricing</v>
+        <v>E06; https://cloud.google.com/vpc/network-pricing</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>ops_labor</v>
+        <v>load_balancer</v>
       </c>
       <c r="B34" t="str">
-        <v>Nhân sự vận hành: 1 FTE SRE/MLOps (trực giờ hành chính, on-call sự cố)</v>
+        <v>Data processing của Load Balancer tại Singapore (vào + ra)</v>
       </c>
       <c r="C34" t="str">
-        <v>1 FTE × 3500 USD/tháng (lương + bảo hiểm + phụ cấp on-call); phụ trách GKE, CI/CD, Terraform, backup, cảnh báo</v>
+        <v>SKU 17FF-00DE-2217 / A9BA-43D3-25AD: (70 GB vào + 200 GB ra) × 0.009 USD/GB. Vào: 1,1 triệu request/tháng × 20 KB + upload file; ra: response stream + asset + file DOCX/XLSX/PPTX</v>
       </c>
       <c r="D34">
-        <v>3500</v>
+        <v>2.43</v>
       </c>
       <c r="E34" t="str">
-        <v>NA</v>
+        <v>E06; https://cloud.google.com/vpc/network-pricing</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>licenses</v>
+        <v>network</v>
       </c>
       <c r="B35" t="str">
-        <v>Gói Google Cloud Customer Care - Standard Support (hỗ trợ kỹ thuật 24/7 cho production)</v>
+        <v>Cloud NAT gateway cho node private gọi API SaaS connectors (kiểm soát egress)</v>
       </c>
       <c r="C35" t="str">
-        <v>max(29 USD; 3% × tổng chi phí cloud các dòng 2-33), công thức tự cập nhật khi nhóm điền đủ</v>
+        <v>SKU 32E2-4EFC-EF9F: 0.0014 USD/VM-giờ × 5260 VM-giờ (app 3×730 + 3×220, staging 1×220, sandbox 3×730). Vertex AI đi qua Private Google Access, không qua NAT</v>
       </c>
       <c r="D35">
-        <f>MAX(29,0.03*(SUM(D2:D33)))</f>
-        <v>29</v>
+        <v>7.36</v>
       </c>
       <c r="E35" t="str">
-        <v>E13; https://cloud.google.com/support</v>
+        <v>E07; https://cloud.google.com/nat/pricing</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>contingency</v>
+        <v>network</v>
       </c>
       <c r="B36" t="str">
-        <v>Dự phòng cho phần biến động theo lượng dùng (token LLM, embedding)</v>
+        <v>IP public của Cloud NAT (IP cố định để SaaS whitelist)</v>
       </c>
       <c r="C36" t="str">
-        <v>10% × (tổng dòng llm + embedding): token/user là ước lượng nên dễ lệch nhất; công thức tự cập nhật</v>
+        <v>SKU 8515-9425-D2CE: 1 IP × 730 giờ × 0.005 USD/giờ</v>
       </c>
       <c r="D36">
-        <f>0.1*(SUMIF(A2:A33,"llm",D2:D33)+SUMIF(A2:A33,"embedding",D2:D33))</f>
-        <v>0</v>
+        <v>3.65</v>
       </c>
       <c r="E36" t="str">
-        <v>NA</v>
+        <v>E07; https://cloud.google.com/nat/pricing</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>network</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Dữ liệu qua Cloud NAT: gọi API Google Workspace, M365, Notion, Jira, Confluence và đồng bộ index</v>
+      </c>
+      <c r="C37" t="str">
+        <v>SKU 015F-5732-FFF0: 300 GB/tháng (vào + ra) × 0.045 USD/GB</v>
+      </c>
+      <c r="D37">
+        <v>13.5</v>
+      </c>
+      <c r="E37" t="str">
+        <v>E07; https://cloud.google.com/nat/pricing</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>network</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Internet egress Premium Tier từ Singapore tới người dùng tại Việt Nam (APAC)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>SKU 400E-0B94-6FB4 (Singapore → APAC, bậc 0-1 TiB): 220 GB × 0.12 USD/GB (200 GB response qua LB + 20 GB request ra SaaS)</v>
+      </c>
+      <c r="D38">
+        <v>26.4</v>
+      </c>
+      <c r="E38" t="str">
+        <v>E08; https://cloud.google.com/vpc/network-pricing</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>network</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Lưu lượng giữa các zone (multi-AZ): pod ↔ pod, pod ↔ Cloud SQL/Redis</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Inter-zone data transfer cùng region, SKU DE9E-AFBC-A15A: 200 GB × 0.01 USD/GB</v>
+      </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39" t="str">
+        <v>E09; https://cloud.google.com/vpc/network-pricing</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>network</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Cloud Armor Standard WAF: chặn SQLi/XSS (OWASP CRS), rate limit theo IP</v>
+      </c>
+      <c r="C40" t="str">
+        <v>1 policy × 5 USD + 4 rule × 1 USD + 15 triệu request × 0.75 USD/triệu (SKU 4B13-E64F-4A2B, A321-89BD-F5BC, 1A87-DEB9-C4BE)</v>
+      </c>
+      <c r="D40">
+        <v>20.25</v>
+      </c>
+      <c r="E40" t="str">
+        <v>E10; https://cloud.google.com/armor/pricing</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>cicd</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Cloud Build: pipeline build/test/deploy lên staging rồi production (IaC Terraform)</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Build time e2-standard-2, SKU A464-9020-6404: 10 service × 2 build/ngày × 22 ngày × 6 phút = 2640 phút × 0.006 USD/phút (tính toàn bộ số phút theo đơn giá niêm yết)</v>
+      </c>
+      <c r="D41">
+        <v>15.84</v>
+      </c>
+      <c r="E41" t="str">
+        <v>E11; https://cloud.google.com/build/pricing</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>cicd</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Artifact Registry: lưu container image cho staging và production</v>
+      </c>
+      <c r="C42" t="str">
+        <v>SKU 8502-299A-ABAF: 30 GB (10 service × ~300 MB × giữ 10 phiên bản, cleanup policy) × 0.1 USD/GB-tháng</v>
+      </c>
+      <c r="D42">
+        <v>3</v>
+      </c>
+      <c r="E42" t="str">
+        <v>E12; https://cloud.google.com/artifact-registry/pricing</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>ops_labor</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Nhân sự vận hành: 1 FTE SRE/MLOps (trực giờ hành chính, on-call sự cố)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>1 FTE × 3500 USD/tháng (lương + bảo hiểm + phụ cấp on-call); phụ trách GKE, CI/CD, Terraform, backup, cảnh báo</v>
+      </c>
+      <c r="D43">
+        <v>3500</v>
+      </c>
+      <c r="E43" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>licenses</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Gói Google Cloud Customer Care - Standard Support (hỗ trợ kỹ thuật 24/7 cho production)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>max(29 USD; 3% × tổng chi phí cloud các dòng 2-42), công thức tự cập nhật khi nhóm điền đủ</v>
+      </c>
+      <c r="D44">
+        <f>MAX(29,0.03*(SUM(D2:D42)))</f>
+        <v>43.35</v>
+      </c>
+      <c r="E44" t="str">
+        <v>E13; https://cloud.google.com/support</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>contingency</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Dự phòng cho phần biến động theo lượng dùng (token LLM, embedding)</v>
+      </c>
+      <c r="C45" t="str">
+        <v>10% × (tổng dòng llm + embedding): token/user là ước lượng nên dễ lệch nhất; công thức tự cập nhật</v>
+      </c>
+      <c r="D45">
+        <f>0.1*(SUMIF(A2:A42,"llm",D2:D42)+SUMIF(A2:A42,"embedding",D2:D42))</f>
+        <v>0</v>
+      </c>
+      <c r="E45" t="str">
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="B37" t="str">
-        <v/>
-      </c>
-      <c r="C37" t="str">
-        <v/>
-      </c>
-      <c r="D37">
-        <f>SUM(D2:D36)</f>
-        <v>4082.99</v>
-      </c>
-      <c r="E37" t="str">
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v/>
+      </c>
+      <c r="D46">
+        <f>SUM(D2:D45)</f>
+        <v>4988.2</v>
+      </c>
+      <c r="E46" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E37"/>
+  <autoFilter ref="A1:E46"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E22"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -1299,9 +1452,145 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>E30</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Cloud SQL for PostgreSQL, Singapore: Regional vCPU 0.1156 USD/giờ, RAM 0.0196 USD/GB-giờ, storage 0.476 USD/GB-tháng; Zonal vCPU 0.0578, RAM 0.0098, storage 0.238 (SKU 0152-2835-C929, 37B4-B2B7-C640, 83A6-DA61-7797, DE86-B401-E60F, EF83-F6A8-8EA7, 45B3-606F-EE91)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>https://cloud.google.com/sql/pricing</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>E31</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Cloud SQL committed use 1 năm, asia-southeast1: 0.0075 USD cho mỗi 0.01 USD/giờ cam kết, tức giảm 25% vCPU + RAM (SKU B4F3-4753-84D8)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>https://cloud.google.com/sql/cud</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>E32</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Cloud Storage Singapore: Standard 0.020, Nearline 0.010 USD/GB-tháng; Class A 0.05 USD/10.000, Class B 0.004 USD/10.000; Nearline Class A 0.10 USD/10.000; Nearline retrieval 0.01 USD/GB (SKU 76BA-5CAD-4338, 4453-FEE4-941B, 4DBF-185F-A415, 7870-010B-2763, 9559-D2EC-1D33, 8D92-97F6-DDF3)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>https://cloud.google.com/storage/pricing</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>E33</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Memorystore for Redis Standard tier, Singapore: M2 (5-10 GB) 0.075 USD/GB-giờ, M1 (1-4 GB) 0.114 USD/GB-giờ (SKU A728-AD0D-27B4, ABC0-67FF-FCAD)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>https://cloud.google.com/memorystore/docs/redis/pricing</v>
+      </c>
+      <c r="D18" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>E34</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Cloud Tasks: 0.40 USD/triệu operation (SKU 378A-D762-1F74)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>https://cloud.google.com/tasks/pricing</v>
+      </c>
+      <c r="D19" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>E35</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Pub/Sub: message delivery 40 USD/TiB, lưu message 0.27 USD/GB-tháng (SKU 027D-B6C7-CCA2, F9EB-D3E1-ABDF)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>https://cloud.google.com/pubsub/pricing</v>
+      </c>
+      <c r="D20" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>E36</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Cloud Scheduler: 0.10 USD/job-tháng = 0.003225806 USD/job-ngày (SKU A5D6-43A2-28A7)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>https://cloud.google.com/scheduler/pricing</v>
+      </c>
+      <c r="D21" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>E37</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Cloud SQL for PostgreSQL hỗ trợ extension pgvector (CREATE EXTENSION vector), không tính phí riêng ngoài instance</v>
+      </c>
+      <c r="C22" t="str">
+        <v>https://cloud.google.com/sql/docs/postgres/work-with-vectors</v>
+      </c>
+      <c r="D22" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>